<commit_message>
Adjuntos reales en todos los casos; las notas se aclaran como Lenguaje
</commit_message>
<xml_diff>
--- a/casos/planilla_6basico_ejemplo.xlsx
+++ b/casos/planilla_6basico_ejemplo.xlsx
@@ -524,7 +524,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Los nombres se reemplazaron por códigos a propósito: a la IA no se le mandan datos de estudiantes.</t>
+          <t>Las tres notas son las evaluaciones de LENGUAJE del semestre, una por mes. Los nombres se reemplazaron por códigos: a la IA no se le mandan datos de estudiantes.</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>NOTAS (1,0 a 7,0)</t>
+          <t>NOTAS DE LENGUAJE (1,0 a 7,0)</t>
         </is>
       </c>
     </row>
@@ -568,17 +568,17 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Nota 1</t>
+          <t>Marzo</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nota 2</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Nota 3</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">

</xml_diff>